<commit_message>
Refresh the product master templates and test them on every run
- Templates: drop the GST Rate, Compensation Cess Rate and HSN Code
  columns (no tax in this project); add Barcode and Net Explosive
  Content (kg), which the importer already reads. The .xlsx gets a
  "How to fill" sheet saying which columns are imported.
- Importer: ignore columns with a blank header; one at the end of the
  old .xlsx was matched to every unmapped field by the auto-mapping.
- Tests import both repository templates and an old-format file with
  tax columns (still imports; those columns are ignored).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DQRBk3XGaHbSWLxgEEj8Hg
</commit_message>
<xml_diff>
--- a/Product_Master_Template.xlsx
+++ b/Product_Master_Template.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Master" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to fill" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +26,25 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +59,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,128 +430,122 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:S6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
     <col width="25" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="28" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
-    <col width="24" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="31" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="28" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Product Code / SKU</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Product Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Subcategory</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Units per Box</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Boxes per Carton</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Units per Carton</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Cost Price</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>MRP</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Retail Selling Price</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Wholesale Selling Price</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>GST Rate</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Compensation Cess Rate</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>HSN Code</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Opening Stock</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>Minimum Stock / Reorder Level</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>Brand / Manufacturer</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>Batch/Lot if available</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Barcode</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>Net Explosive Content (kg)</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>Product Status</t>
         </is>
@@ -588,33 +599,30 @@
         <v>85</v>
       </c>
       <c r="M2" t="n">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>3604</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>10</v>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
           <t>Sample Brand</t>
         </is>
       </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>B001</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>8901234500017</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>0.05</v>
+      </c>
       <c r="S2" t="inlineStr">
-        <is>
-          <t>B001</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -668,33 +676,26 @@
         <v>150</v>
       </c>
       <c r="M3" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>3604</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>30</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>5</v>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
           <t>Sample Brand</t>
         </is>
       </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>B002</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr"/>
+      <c r="R3" t="n">
+        <v>0.25</v>
+      </c>
       <c r="S3" t="inlineStr">
-        <is>
-          <t>B002</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -748,33 +749,26 @@
         <v>300</v>
       </c>
       <c r="M4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>3604</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>5</v>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
           <t>Sample Brand</t>
         </is>
       </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>B003</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr"/>
+      <c r="R4" t="n">
+        <v>0.5</v>
+      </c>
       <c r="S4" t="inlineStr">
-        <is>
-          <t>B003</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -828,33 +822,26 @@
         <v>115</v>
       </c>
       <c r="M5" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>3604</t>
-        </is>
-      </c>
-      <c r="P5" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>5</v>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
           <t>Sample Brand</t>
         </is>
       </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>B004</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr"/>
+      <c r="R5" t="n">
+        <v>0.1</v>
+      </c>
       <c r="S5" t="inlineStr">
-        <is>
-          <t>B004</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -908,35 +895,113 @@
         <v>820</v>
       </c>
       <c r="M6" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="N6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>3604</t>
-        </is>
-      </c>
-      <c r="P6" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>3</v>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
           <t>Sample Brand</t>
         </is>
       </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>B005</t>
+        </is>
+      </c>
+      <c r="Q6" s="3" t="inlineStr"/>
+      <c r="R6" t="n">
+        <v>1.2</v>
+      </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>B005</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
           <t>ACTIVE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Product Master import - how to fill the first sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Product Code / SKU (unique), Product Name, Retail Selling Price (yellow headers)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Used by the app</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Category, Subcategory, Unit, Cost Price (profit reports), Opening Stock, Minimum Stock / Reorder Level, Brand / Manufacturer, Barcode, Net Explosive Content (kg) per unit (licence storage limit), Product Status (ACTIVE or INACTIVE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>For your records only</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Units per Box, Boxes per Carton, Units per Carton, MRP, Wholesale Selling Price, Batch/Lot - kept in this file, not imported</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Rules</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Upload in Products -&gt; Upload Product Master. You can map columns with other names. If any row has a problem nothing is imported; fix the rows listed and upload again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Only the first sheet is read. Keep one header row. Prices and stock must not be negative.</t>
         </is>
       </c>
     </row>

</xml_diff>